<commit_message>
run for insight 2025 update
</commit_message>
<xml_diff>
--- a/output_data/charts/capacity-15-CountyRegion-M010000US001.xlsx
+++ b/output_data/charts/capacity-15-CountyRegion-M010000US001.xlsx
@@ -167,10 +167,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="23"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -178,72 +178,66 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2002</c:v>
+                  <c:v>2004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2003</c:v>
+                  <c:v>2005</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2004</c:v>
+                  <c:v>2006</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2005</c:v>
+                  <c:v>2007</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2006</c:v>
+                  <c:v>2008</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2007</c:v>
+                  <c:v>2009</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2008</c:v>
+                  <c:v>2010</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2009</c:v>
+                  <c:v>2011</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2010</c:v>
+                  <c:v>2012</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2011</c:v>
+                  <c:v>2013</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2012</c:v>
+                  <c:v>2014</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2013</c:v>
+                  <c:v>2015</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2014</c:v>
+                  <c:v>2016</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2015</c:v>
+                  <c:v>2017</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2016</c:v>
+                  <c:v>2018</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2017</c:v>
+                  <c:v>2019</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2018</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2019</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2020</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2021</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2022</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -251,84 +245,12 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$26</c:f>
+              <c:f>Sheet1!$B$2:$B$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
+                <c:ptCount val="23"/>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="13">
                   <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -358,10 +280,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="23"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -369,72 +291,66 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2002</c:v>
+                  <c:v>2004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2003</c:v>
+                  <c:v>2005</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2004</c:v>
+                  <c:v>2006</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2005</c:v>
+                  <c:v>2007</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2006</c:v>
+                  <c:v>2008</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2007</c:v>
+                  <c:v>2009</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2008</c:v>
+                  <c:v>2010</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2009</c:v>
+                  <c:v>2011</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2010</c:v>
+                  <c:v>2012</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2011</c:v>
+                  <c:v>2013</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2012</c:v>
+                  <c:v>2014</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2013</c:v>
+                  <c:v>2015</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2014</c:v>
+                  <c:v>2016</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2015</c:v>
+                  <c:v>2017</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2016</c:v>
+                  <c:v>2018</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2017</c:v>
+                  <c:v>2019</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2018</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2019</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2020</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2021</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2022</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -442,84 +358,33 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$2:$C$26</c:f>
+              <c:f>Sheet1!$C$2:$C$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
+                <c:ptCount val="23"/>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="13">
                   <c:v>4000</c:v>
                 </c:pt>
-                <c:pt idx="14">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>100</c:v>
+                  <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0</c:v>
+                  <c:v>600</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>250</c:v>
+                  <c:v>78.28</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>600</c:v>
+                  <c:v>142.76</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>78.28</c:v>
+                  <c:v>438.67</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>132.76</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>438.67</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>1642.24</c:v>
+                  <c:v>1657.24</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -549,10 +414,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="23"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -560,72 +425,66 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2002</c:v>
+                  <c:v>2004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2003</c:v>
+                  <c:v>2005</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2004</c:v>
+                  <c:v>2006</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2005</c:v>
+                  <c:v>2007</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2006</c:v>
+                  <c:v>2008</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2007</c:v>
+                  <c:v>2009</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2008</c:v>
+                  <c:v>2010</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2009</c:v>
+                  <c:v>2011</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2010</c:v>
+                  <c:v>2012</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2011</c:v>
+                  <c:v>2013</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2012</c:v>
+                  <c:v>2014</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2013</c:v>
+                  <c:v>2015</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2014</c:v>
+                  <c:v>2016</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2015</c:v>
+                  <c:v>2017</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2016</c:v>
+                  <c:v>2018</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2017</c:v>
+                  <c:v>2019</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2018</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2019</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2020</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2021</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2022</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -633,84 +492,18 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$26</c:f>
+              <c:f>Sheet1!$D$2:$D$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0</c:v>
-                </c:pt>
+                <c:ptCount val="23"/>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>248</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="18">
                   <c:v>15036</c:v>
                 </c:pt>
-                <c:pt idx="19">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="21">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="23">
                   <c:v>4804</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -740,10 +533,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="23"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -751,72 +544,66 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2002</c:v>
+                  <c:v>2004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2003</c:v>
+                  <c:v>2005</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2004</c:v>
+                  <c:v>2006</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2005</c:v>
+                  <c:v>2007</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2006</c:v>
+                  <c:v>2008</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2007</c:v>
+                  <c:v>2009</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2008</c:v>
+                  <c:v>2010</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2009</c:v>
+                  <c:v>2011</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2010</c:v>
+                  <c:v>2012</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2011</c:v>
+                  <c:v>2013</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2012</c:v>
+                  <c:v>2014</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2013</c:v>
+                  <c:v>2015</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2014</c:v>
+                  <c:v>2016</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2015</c:v>
+                  <c:v>2017</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2016</c:v>
+                  <c:v>2018</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2017</c:v>
+                  <c:v>2019</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2018</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2019</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2020</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2021</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2022</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -824,84 +611,69 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$2:$E$26</c:f>
+              <c:f>Sheet1!$E$2:$E$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
+                <c:ptCount val="23"/>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>1.65</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>13.86</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.65</c:v>
+                  <c:v>32.65</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>13.86</c:v>
+                  <c:v>69.3</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>25.05</c:v>
+                  <c:v>77.40000000000001</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>69.3</c:v>
+                  <c:v>515.23</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>77.40000000000001</c:v>
+                  <c:v>1817.347</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>445.49</c:v>
+                  <c:v>6857.23</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1305.165</c:v>
+                  <c:v>1690.355</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>6853.46</c:v>
+                  <c:v>2255.857</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1690.355</c:v>
+                  <c:v>1443.925</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2244.24</c:v>
+                  <c:v>1664.465</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1399.48</c:v>
+                  <c:v>4970.52</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1373.165</c:v>
+                  <c:v>2583.925</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4905.78</c:v>
+                  <c:v>15187.31</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2522.11</c:v>
+                  <c:v>5012.295</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>6608.96</c:v>
+                  <c:v>8628.021999999999</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>4931.88</c:v>
+                  <c:v>10548.826</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>8517.262000000001</c:v>
+                  <c:v>23815.572</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>10409.82</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>23790.902</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>20800.418</c:v>
+                  <c:v>20798.506</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -931,10 +703,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="23"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -942,72 +714,66 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2002</c:v>
+                  <c:v>2004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2003</c:v>
+                  <c:v>2005</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2004</c:v>
+                  <c:v>2006</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2005</c:v>
+                  <c:v>2007</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2006</c:v>
+                  <c:v>2008</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2007</c:v>
+                  <c:v>2009</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2008</c:v>
+                  <c:v>2010</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2009</c:v>
+                  <c:v>2011</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2010</c:v>
+                  <c:v>2012</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2011</c:v>
+                  <c:v>2013</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2012</c:v>
+                  <c:v>2014</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2013</c:v>
+                  <c:v>2015</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2014</c:v>
+                  <c:v>2016</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2015</c:v>
+                  <c:v>2017</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2016</c:v>
+                  <c:v>2018</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2017</c:v>
+                  <c:v>2019</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2018</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2019</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2020</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2021</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2022</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -1015,84 +781,12 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$2:$F$26</c:f>
+              <c:f>Sheet1!$F$2:$F$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0</c:v>
-                </c:pt>
+                <c:ptCount val="23"/>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="17">
                   <c:v>3500</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1122,10 +816,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="23"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -1133,72 +827,66 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2002</c:v>
+                  <c:v>2004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2003</c:v>
+                  <c:v>2005</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2004</c:v>
+                  <c:v>2006</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2005</c:v>
+                  <c:v>2007</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2006</c:v>
+                  <c:v>2008</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2007</c:v>
+                  <c:v>2009</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2008</c:v>
+                  <c:v>2010</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2009</c:v>
+                  <c:v>2011</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2010</c:v>
+                  <c:v>2012</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2011</c:v>
+                  <c:v>2013</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2012</c:v>
+                  <c:v>2014</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2013</c:v>
+                  <c:v>2015</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2014</c:v>
+                  <c:v>2016</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2015</c:v>
+                  <c:v>2017</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2016</c:v>
+                  <c:v>2018</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2017</c:v>
+                  <c:v>2019</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2018</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2019</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2020</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2021</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2022</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -1206,10 +894,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$2:$G$26</c:f>
+              <c:f>Sheet1!$G$2:$G$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="23"/>
                 <c:pt idx="0">
                   <c:v>10</c:v>
                 </c:pt>
@@ -1217,73 +905,31 @@
                   <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>1.8</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>47.8</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.8</c:v>
+                  <c:v>161.8</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>47.8</c:v>
+                  <c:v>2.4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>161.8</c:v>
+                  <c:v>1.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.4</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>1.5</c:v>
-                </c:pt>
-                <c:pt idx="13">
                   <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="14">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="16">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="18">
                   <c:v>4500</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1714,7 +1360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
@@ -1753,21 +1399,6 @@
       <c r="A2" s="3">
         <v>2000</v>
       </c>
-      <c r="B2" s="2">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
-        <v>0</v>
-      </c>
-      <c r="F2" s="2">
-        <v>0</v>
-      </c>
       <c r="G2" s="2">
         <v>10</v>
       </c>
@@ -1776,552 +1407,239 @@
       <c r="A3" s="3">
         <v>2001</v>
       </c>
-      <c r="B3" s="2">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
-        <v>0</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0</v>
-      </c>
       <c r="G3" s="2">
         <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="3">
-        <v>2002</v>
-      </c>
-      <c r="B4" s="2">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2">
-        <v>0</v>
-      </c>
-      <c r="F4" s="2">
-        <v>0</v>
+        <v>2004</v>
       </c>
       <c r="G4" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="3">
-        <v>2003</v>
-      </c>
-      <c r="B5" s="2">
-        <v>0</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0</v>
+        <v>2005</v>
       </c>
       <c r="E5" s="2">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2">
-        <v>0</v>
+        <v>1.65</v>
       </c>
       <c r="G5" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="3">
-        <v>2004</v>
-      </c>
-      <c r="B6" s="2">
-        <v>0</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0</v>
+        <v>2006</v>
       </c>
       <c r="E6" s="2">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2">
-        <v>0</v>
-      </c>
-      <c r="G6" s="2">
-        <v>1</v>
+        <v>13.86</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="3">
-        <v>2005</v>
-      </c>
-      <c r="B7" s="2">
-        <v>0</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0</v>
+        <v>2007</v>
       </c>
       <c r="E7" s="2">
-        <v>1.65</v>
-      </c>
-      <c r="F7" s="2">
-        <v>0</v>
-      </c>
-      <c r="G7" s="2">
-        <v>8</v>
+        <v>32.65</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="3">
-        <v>2006</v>
-      </c>
-      <c r="B8" s="2">
-        <v>0</v>
-      </c>
-      <c r="C8" s="2">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0</v>
+        <v>2008</v>
       </c>
       <c r="E8" s="2">
-        <v>13.86</v>
-      </c>
-      <c r="F8" s="2">
-        <v>0</v>
+        <v>69.3</v>
       </c>
       <c r="G8" s="2">
-        <v>0</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="3">
-        <v>2007</v>
-      </c>
-      <c r="B9" s="2">
-        <v>0</v>
-      </c>
-      <c r="C9" s="2">
-        <v>0</v>
-      </c>
-      <c r="D9" s="2">
-        <v>0</v>
+        <v>2009</v>
       </c>
       <c r="E9" s="2">
-        <v>25.05</v>
-      </c>
-      <c r="F9" s="2">
-        <v>0</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="G9" s="2">
-        <v>0</v>
+        <v>47.8</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="3">
-        <v>2008</v>
-      </c>
-      <c r="B10" s="2">
-        <v>0</v>
-      </c>
-      <c r="C10" s="2">
-        <v>0</v>
-      </c>
-      <c r="D10" s="2">
-        <v>0</v>
+        <v>2010</v>
       </c>
       <c r="E10" s="2">
-        <v>69.3</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0</v>
+        <v>515.23</v>
       </c>
       <c r="G10" s="2">
-        <v>1.8</v>
+        <v>161.8</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="3">
-        <v>2009</v>
-      </c>
-      <c r="B11" s="2">
-        <v>0</v>
-      </c>
-      <c r="C11" s="2">
-        <v>0</v>
-      </c>
-      <c r="D11" s="2">
-        <v>0</v>
+        <v>2011</v>
       </c>
       <c r="E11" s="2">
-        <v>77.40000000000001</v>
-      </c>
-      <c r="F11" s="2">
-        <v>0</v>
+        <v>1817.347</v>
       </c>
       <c r="G11" s="2">
-        <v>47.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="3">
-        <v>2010</v>
-      </c>
-      <c r="B12" s="2">
-        <v>0</v>
-      </c>
-      <c r="C12" s="2">
-        <v>0</v>
-      </c>
-      <c r="D12" s="2">
-        <v>0</v>
+        <v>2012</v>
       </c>
       <c r="E12" s="2">
-        <v>445.49</v>
-      </c>
-      <c r="F12" s="2">
-        <v>0</v>
+        <v>6857.23</v>
       </c>
       <c r="G12" s="2">
-        <v>161.8</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="3">
-        <v>2011</v>
+        <v>2013</v>
       </c>
       <c r="B13" s="2">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="C13" s="2">
-        <v>0</v>
-      </c>
-      <c r="D13" s="2">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="E13" s="2">
-        <v>1305.165</v>
-      </c>
-      <c r="F13" s="2">
-        <v>0</v>
+        <v>1690.355</v>
       </c>
       <c r="G13" s="2">
-        <v>2.4</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="3">
-        <v>2012</v>
-      </c>
-      <c r="B14" s="2">
-        <v>0</v>
-      </c>
-      <c r="C14" s="2">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2">
-        <v>0</v>
+        <v>2014</v>
       </c>
       <c r="E14" s="2">
-        <v>6853.46</v>
-      </c>
-      <c r="F14" s="2">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2">
-        <v>1.5</v>
+        <v>2255.857</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="3">
-        <v>2013</v>
-      </c>
-      <c r="B15" s="2">
-        <v>400</v>
-      </c>
-      <c r="C15" s="2">
-        <v>4000</v>
+        <v>2015</v>
       </c>
       <c r="D15" s="2">
-        <v>0</v>
+        <v>248</v>
       </c>
       <c r="E15" s="2">
-        <v>1690.355</v>
-      </c>
-      <c r="F15" s="2">
-        <v>0</v>
-      </c>
-      <c r="G15" s="2">
-        <v>30</v>
+        <v>1443.925</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="3">
-        <v>2014</v>
-      </c>
-      <c r="B16" s="2">
-        <v>0</v>
-      </c>
-      <c r="C16" s="2">
-        <v>0</v>
-      </c>
-      <c r="D16" s="2">
-        <v>0</v>
+        <v>2016</v>
       </c>
       <c r="E16" s="2">
-        <v>2244.24</v>
-      </c>
-      <c r="F16" s="2">
-        <v>0</v>
-      </c>
-      <c r="G16" s="2">
-        <v>0</v>
+        <v>1664.465</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="3">
-        <v>2015</v>
-      </c>
-      <c r="B17" s="2">
-        <v>0</v>
+        <v>2017</v>
       </c>
       <c r="C17" s="2">
-        <v>0</v>
-      </c>
-      <c r="D17" s="2">
-        <v>248</v>
+        <v>100</v>
       </c>
       <c r="E17" s="2">
-        <v>1399.48</v>
+        <v>4970.52</v>
       </c>
       <c r="F17" s="2">
-        <v>0</v>
-      </c>
-      <c r="G17" s="2">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="3">
-        <v>2016</v>
-      </c>
-      <c r="B18" s="2">
-        <v>0</v>
-      </c>
-      <c r="C18" s="2">
-        <v>0</v>
+        <v>2018</v>
       </c>
       <c r="D18" s="2">
-        <v>0</v>
+        <v>15036</v>
       </c>
       <c r="E18" s="2">
-        <v>1373.165</v>
-      </c>
-      <c r="F18" s="2">
-        <v>0</v>
+        <v>2583.925</v>
       </c>
       <c r="G18" s="2">
-        <v>0</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="3">
-        <v>2017</v>
-      </c>
-      <c r="B19" s="2">
-        <v>0</v>
+        <v>2019</v>
       </c>
       <c r="C19" s="2">
-        <v>100</v>
-      </c>
-      <c r="D19" s="2">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E19" s="2">
-        <v>4905.78</v>
-      </c>
-      <c r="F19" s="2">
-        <v>3500</v>
-      </c>
-      <c r="G19" s="2">
-        <v>0</v>
+        <v>15187.31</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="3">
-        <v>2018</v>
-      </c>
-      <c r="B20" s="2">
-        <v>0</v>
+        <v>2020</v>
       </c>
       <c r="C20" s="2">
-        <v>0</v>
-      </c>
-      <c r="D20" s="2">
-        <v>15036</v>
+        <v>600</v>
       </c>
       <c r="E20" s="2">
-        <v>2522.11</v>
-      </c>
-      <c r="F20" s="2">
-        <v>0</v>
-      </c>
-      <c r="G20" s="2">
-        <v>4500</v>
+        <v>5012.295</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="3">
-        <v>2019</v>
-      </c>
-      <c r="B21" s="2">
-        <v>0</v>
+        <v>2021</v>
       </c>
       <c r="C21" s="2">
-        <v>250</v>
-      </c>
-      <c r="D21" s="2">
-        <v>0</v>
+        <v>78.28</v>
       </c>
       <c r="E21" s="2">
-        <v>6608.96</v>
-      </c>
-      <c r="F21" s="2">
-        <v>0</v>
-      </c>
-      <c r="G21" s="2">
-        <v>0</v>
+        <v>8628.021999999999</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="3">
-        <v>2020</v>
-      </c>
-      <c r="B22" s="2">
-        <v>0</v>
+        <v>2022</v>
       </c>
       <c r="C22" s="2">
-        <v>600</v>
-      </c>
-      <c r="D22" s="2">
-        <v>0</v>
+        <v>142.76</v>
       </c>
       <c r="E22" s="2">
-        <v>4931.88</v>
-      </c>
-      <c r="F22" s="2">
-        <v>0</v>
-      </c>
-      <c r="G22" s="2">
-        <v>0</v>
+        <v>10548.826</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="3">
-        <v>2021</v>
-      </c>
-      <c r="B23" s="2">
-        <v>0</v>
+        <v>2023</v>
       </c>
       <c r="C23" s="2">
-        <v>78.28</v>
+        <v>438.67</v>
       </c>
       <c r="D23" s="2">
-        <v>0</v>
+        <v>4804</v>
       </c>
       <c r="E23" s="2">
-        <v>8517.262000000001</v>
-      </c>
-      <c r="F23" s="2">
-        <v>0</v>
-      </c>
-      <c r="G23" s="2">
-        <v>0</v>
+        <v>23815.572</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="3">
-        <v>2022</v>
-      </c>
-      <c r="B24" s="2">
-        <v>0</v>
+        <v>2024</v>
       </c>
       <c r="C24" s="2">
-        <v>132.76</v>
-      </c>
-      <c r="D24" s="2">
-        <v>0</v>
+        <v>1657.24</v>
       </c>
       <c r="E24" s="2">
-        <v>10409.82</v>
-      </c>
-      <c r="F24" s="2">
-        <v>0</v>
-      </c>
-      <c r="G24" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="3">
-        <v>2023</v>
-      </c>
-      <c r="B25" s="2">
-        <v>0</v>
-      </c>
-      <c r="C25" s="2">
-        <v>438.67</v>
-      </c>
-      <c r="D25" s="2">
-        <v>4804</v>
-      </c>
-      <c r="E25" s="2">
-        <v>23790.902</v>
-      </c>
-      <c r="F25" s="2">
-        <v>0</v>
-      </c>
-      <c r="G25" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26" s="3">
-        <v>2024</v>
-      </c>
-      <c r="B26" s="2">
-        <v>0</v>
-      </c>
-      <c r="C26" s="2">
-        <v>1642.24</v>
-      </c>
-      <c r="D26" s="2">
-        <v>0</v>
-      </c>
-      <c r="E26" s="2">
-        <v>20800.418</v>
-      </c>
-      <c r="F26" s="2">
-        <v>0</v>
-      </c>
-      <c r="G26" s="2">
-        <v>0</v>
+        <v>20798.506</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correct charts x-axis to include all years
</commit_message>
<xml_diff>
--- a/output_data/charts/capacity-15-CountyRegion-M010000US001.xlsx
+++ b/output_data/charts/capacity-15-CountyRegion-M010000US001.xlsx
@@ -167,10 +167,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$24</c:f>
+              <c:f>Sheet1!$A$2:$A$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="25"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -178,66 +178,72 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>2002</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2003</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>2004</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>2005</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>2006</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
                   <c:v>2007</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>2008</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>2009</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>2010</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
                   <c:v>2011</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
                   <c:v>2012</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="13">
                   <c:v>2013</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="14">
                   <c:v>2014</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="15">
                   <c:v>2015</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>2016</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>2017</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>2018</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>2019</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="20">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="21">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="22">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="23">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -245,11 +251,11 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$24</c:f>
+              <c:f>Sheet1!$B$2:$B$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
-                <c:pt idx="11">
+                <c:ptCount val="25"/>
+                <c:pt idx="13">
                   <c:v>400</c:v>
                 </c:pt>
               </c:numCache>
@@ -280,10 +286,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$24</c:f>
+              <c:f>Sheet1!$A$2:$A$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="25"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -291,66 +297,72 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>2002</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2003</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>2004</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>2005</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>2006</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
                   <c:v>2007</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>2008</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>2009</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>2010</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
                   <c:v>2011</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
                   <c:v>2012</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="13">
                   <c:v>2013</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="14">
                   <c:v>2014</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="15">
                   <c:v>2015</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>2016</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>2017</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>2018</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>2019</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="20">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="21">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="22">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="23">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -358,32 +370,32 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$2:$C$24</c:f>
+              <c:f>Sheet1!$C$2:$C$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
-                <c:pt idx="11">
+                <c:ptCount val="25"/>
+                <c:pt idx="13">
                   <c:v>4000</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>250</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="20">
                   <c:v>600</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="21">
                   <c:v>78.28</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="22">
                   <c:v>142.76</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="23">
                   <c:v>438.67</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="24">
                   <c:v>1657.24</c:v>
                 </c:pt>
               </c:numCache>
@@ -414,10 +426,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$24</c:f>
+              <c:f>Sheet1!$A$2:$A$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="25"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -425,66 +437,72 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>2002</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2003</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>2004</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>2005</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>2006</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
                   <c:v>2007</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>2008</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>2009</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>2010</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
                   <c:v>2011</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
                   <c:v>2012</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="13">
                   <c:v>2013</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="14">
                   <c:v>2014</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="15">
                   <c:v>2015</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>2016</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>2017</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>2018</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>2019</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="20">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="21">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="22">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="23">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -492,17 +510,17 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$24</c:f>
+              <c:f>Sheet1!$D$2:$D$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
-                <c:pt idx="13">
+                <c:ptCount val="25"/>
+                <c:pt idx="15">
                   <c:v>248</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>15036</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="23">
                   <c:v>4804</c:v>
                 </c:pt>
               </c:numCache>
@@ -533,10 +551,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$24</c:f>
+              <c:f>Sheet1!$A$2:$A$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="25"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -544,66 +562,72 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>2002</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2003</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>2004</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>2005</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>2006</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
                   <c:v>2007</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>2008</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>2009</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>2010</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
                   <c:v>2011</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
                   <c:v>2012</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="13">
                   <c:v>2013</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="14">
                   <c:v>2014</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="15">
                   <c:v>2015</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>2016</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>2017</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>2018</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>2019</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="20">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="21">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="22">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="23">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -611,68 +635,68 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$2:$E$24</c:f>
+              <c:f>Sheet1!$E$2:$E$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
-                <c:pt idx="3">
+                <c:ptCount val="25"/>
+                <c:pt idx="5">
                   <c:v>1.65</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>13.86</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
                   <c:v>32.65</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>69.3</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>77.40000000000001</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>515.23</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
                   <c:v>1817.347</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
                   <c:v>6857.23</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="13">
                   <c:v>1690.355</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="14">
                   <c:v>2255.857</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="15">
                   <c:v>1443.925</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>1664.465</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>4970.52</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>2583.925</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>15187.31</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="20">
                   <c:v>5012.295</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="21">
                   <c:v>8628.021999999999</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="22">
                   <c:v>10548.826</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="23">
                   <c:v>23815.572</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="24">
                   <c:v>20798.506</c:v>
                 </c:pt>
               </c:numCache>
@@ -703,10 +727,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$24</c:f>
+              <c:f>Sheet1!$A$2:$A$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="25"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -714,66 +738,72 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>2002</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2003</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>2004</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>2005</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>2006</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
                   <c:v>2007</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>2008</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>2009</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>2010</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
                   <c:v>2011</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
                   <c:v>2012</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="13">
                   <c:v>2013</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="14">
                   <c:v>2014</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="15">
                   <c:v>2015</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>2016</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>2017</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>2018</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>2019</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="20">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="21">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="22">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="23">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -781,11 +811,11 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$2:$F$24</c:f>
+              <c:f>Sheet1!$F$2:$F$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
-                <c:pt idx="15">
+                <c:ptCount val="25"/>
+                <c:pt idx="17">
                   <c:v>3500</c:v>
                 </c:pt>
               </c:numCache>
@@ -816,10 +846,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$24</c:f>
+              <c:f>Sheet1!$A$2:$A$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="25"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -827,66 +857,72 @@
                   <c:v>2001</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>2002</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2003</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>2004</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>2005</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>2006</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
                   <c:v>2007</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>2008</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>2009</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>2010</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
                   <c:v>2011</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
                   <c:v>2012</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="13">
                   <c:v>2013</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="14">
                   <c:v>2014</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="15">
                   <c:v>2015</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>2016</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>2017</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>2018</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>2019</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="20">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="21">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="22">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="23">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="24">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -894,41 +930,41 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$2:$G$24</c:f>
+              <c:f>Sheet1!$G$2:$G$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="25"/>
                 <c:pt idx="0">
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>18</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="4">
                   <c:v>1</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>8</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>1.8</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>47.8</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>161.8</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
                   <c:v>2.4</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
                   <c:v>1.5</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="13">
                   <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>4500</c:v>
                 </c:pt>
               </c:numCache>
@@ -1360,7 +1396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
@@ -1413,232 +1449,242 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="3">
-        <v>2004</v>
-      </c>
-      <c r="G4" s="2">
-        <v>1</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="3">
-        <v>2005</v>
-      </c>
-      <c r="E5" s="2">
-        <v>1.65</v>
-      </c>
-      <c r="G5" s="2">
-        <v>8</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="3">
-        <v>2006</v>
-      </c>
-      <c r="E6" s="2">
-        <v>13.86</v>
+        <v>2004</v>
+      </c>
+      <c r="G6" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="3">
-        <v>2007</v>
+        <v>2005</v>
       </c>
       <c r="E7" s="2">
-        <v>32.65</v>
+        <v>1.65</v>
+      </c>
+      <c r="G7" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="3">
-        <v>2008</v>
+        <v>2006</v>
       </c>
       <c r="E8" s="2">
-        <v>69.3</v>
-      </c>
-      <c r="G8" s="2">
-        <v>1.8</v>
+        <v>13.86</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="3">
-        <v>2009</v>
+        <v>2007</v>
       </c>
       <c r="E9" s="2">
-        <v>77.40000000000001</v>
-      </c>
-      <c r="G9" s="2">
-        <v>47.8</v>
+        <v>32.65</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="3">
-        <v>2010</v>
+        <v>2008</v>
       </c>
       <c r="E10" s="2">
-        <v>515.23</v>
+        <v>69.3</v>
       </c>
       <c r="G10" s="2">
-        <v>161.8</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="3">
-        <v>2011</v>
+        <v>2009</v>
       </c>
       <c r="E11" s="2">
-        <v>1817.347</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="G11" s="2">
-        <v>2.4</v>
+        <v>47.8</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="3">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="E12" s="2">
-        <v>6857.23</v>
+        <v>515.23</v>
       </c>
       <c r="G12" s="2">
-        <v>1.5</v>
+        <v>161.8</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="3">
-        <v>2013</v>
-      </c>
-      <c r="B13" s="2">
-        <v>400</v>
-      </c>
-      <c r="C13" s="2">
-        <v>4000</v>
+        <v>2011</v>
       </c>
       <c r="E13" s="2">
-        <v>1690.355</v>
+        <v>1817.347</v>
       </c>
       <c r="G13" s="2">
-        <v>30</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="3">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="E14" s="2">
-        <v>2255.857</v>
+        <v>6857.23</v>
+      </c>
+      <c r="G14" s="2">
+        <v>1.5</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="3">
-        <v>2015</v>
-      </c>
-      <c r="D15" s="2">
-        <v>248</v>
+        <v>2013</v>
+      </c>
+      <c r="B15" s="2">
+        <v>400</v>
+      </c>
+      <c r="C15" s="2">
+        <v>4000</v>
       </c>
       <c r="E15" s="2">
-        <v>1443.925</v>
+        <v>1690.355</v>
+      </c>
+      <c r="G15" s="2">
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="3">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="E16" s="2">
-        <v>1664.465</v>
+        <v>2255.857</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="3">
-        <v>2017</v>
-      </c>
-      <c r="C17" s="2">
-        <v>100</v>
+        <v>2015</v>
+      </c>
+      <c r="D17" s="2">
+        <v>248</v>
       </c>
       <c r="E17" s="2">
-        <v>4970.52</v>
-      </c>
-      <c r="F17" s="2">
-        <v>3500</v>
+        <v>1443.925</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="3">
-        <v>2018</v>
-      </c>
-      <c r="D18" s="2">
-        <v>15036</v>
+        <v>2016</v>
       </c>
       <c r="E18" s="2">
-        <v>2583.925</v>
-      </c>
-      <c r="G18" s="2">
-        <v>4500</v>
+        <v>1664.465</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="3">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="C19" s="2">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="E19" s="2">
-        <v>15187.31</v>
+        <v>4970.52</v>
+      </c>
+      <c r="F19" s="2">
+        <v>3500</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="3">
-        <v>2020</v>
-      </c>
-      <c r="C20" s="2">
-        <v>600</v>
+        <v>2018</v>
+      </c>
+      <c r="D20" s="2">
+        <v>15036</v>
       </c>
       <c r="E20" s="2">
-        <v>5012.295</v>
+        <v>2583.925</v>
+      </c>
+      <c r="G20" s="2">
+        <v>4500</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="3">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C21" s="2">
-        <v>78.28</v>
+        <v>250</v>
       </c>
       <c r="E21" s="2">
-        <v>8628.021999999999</v>
+        <v>15187.31</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="3">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C22" s="2">
-        <v>142.76</v>
+        <v>600</v>
       </c>
       <c r="E22" s="2">
-        <v>10548.826</v>
+        <v>5012.295</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="3">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C23" s="2">
-        <v>438.67</v>
-      </c>
-      <c r="D23" s="2">
-        <v>4804</v>
+        <v>78.28</v>
       </c>
       <c r="E23" s="2">
-        <v>23815.572</v>
+        <v>8628.021999999999</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="3">
+        <v>2022</v>
+      </c>
+      <c r="C24" s="2">
+        <v>142.76</v>
+      </c>
+      <c r="E24" s="2">
+        <v>10548.826</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="3">
+        <v>2023</v>
+      </c>
+      <c r="C25" s="2">
+        <v>438.67</v>
+      </c>
+      <c r="D25" s="2">
+        <v>4804</v>
+      </c>
+      <c r="E25" s="2">
+        <v>23815.572</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="3">
         <v>2024</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C26" s="2">
         <v>1657.24</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E26" s="2">
         <v>20798.506</v>
       </c>
     </row>

</xml_diff>

<commit_message>
rerun full pipline for der, add 2025 data
</commit_message>
<xml_diff>
--- a/output_data/charts/capacity-15-CountyRegion-M010000US001.xlsx
+++ b/output_data/charts/capacity-15-CountyRegion-M010000US001.xlsx
@@ -255,9 +255,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="25"/>
-                <c:pt idx="13">
-                  <c:v>400</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -374,30 +371,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="25"/>
-                <c:pt idx="13">
-                  <c:v>4000</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>600</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>78.28</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>142.76</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>438.67</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>1657.24</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -514,15 +487,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="25"/>
-                <c:pt idx="15">
-                  <c:v>248</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>15036</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>4804</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -639,66 +603,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="25"/>
-                <c:pt idx="5">
-                  <c:v>1.65</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>13.86</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>32.65</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>69.3</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>77.40000000000001</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>515.23</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1817.347</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>6857.23</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>1690.355</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>2255.857</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>1443.925</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>1664.465</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>4970.52</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>2583.925</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>15187.31</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>5012.295</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>8628.021999999999</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>10548.826</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>23815.572</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>20798.506</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -815,9 +719,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="25"/>
-                <c:pt idx="17">
-                  <c:v>3500</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -934,39 +835,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="25"/>
-                <c:pt idx="0">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>18</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>47.8</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>161.8</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>2.4</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>1.5</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>4500</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1435,17 +1303,11 @@
       <c r="A2" s="3">
         <v>2000</v>
       </c>
-      <c r="G2" s="2">
-        <v>10</v>
-      </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3">
         <v>2001</v>
       </c>
-      <c r="G3" s="2">
-        <v>18</v>
-      </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="3">
@@ -1461,231 +1323,105 @@
       <c r="A6" s="3">
         <v>2004</v>
       </c>
-      <c r="G6" s="2">
-        <v>1</v>
-      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="3">
         <v>2005</v>
       </c>
-      <c r="E7" s="2">
-        <v>1.65</v>
-      </c>
-      <c r="G7" s="2">
-        <v>8</v>
-      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="3">
         <v>2006</v>
       </c>
-      <c r="E8" s="2">
-        <v>13.86</v>
-      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="3">
         <v>2007</v>
       </c>
-      <c r="E9" s="2">
-        <v>32.65</v>
-      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="3">
         <v>2008</v>
       </c>
-      <c r="E10" s="2">
-        <v>69.3</v>
-      </c>
-      <c r="G10" s="2">
-        <v>1.8</v>
-      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="3">
         <v>2009</v>
       </c>
-      <c r="E11" s="2">
-        <v>77.40000000000001</v>
-      </c>
-      <c r="G11" s="2">
-        <v>47.8</v>
-      </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="3">
         <v>2010</v>
       </c>
-      <c r="E12" s="2">
-        <v>515.23</v>
-      </c>
-      <c r="G12" s="2">
-        <v>161.8</v>
-      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="3">
         <v>2011</v>
       </c>
-      <c r="E13" s="2">
-        <v>1817.347</v>
-      </c>
-      <c r="G13" s="2">
-        <v>2.4</v>
-      </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="3">
         <v>2012</v>
       </c>
-      <c r="E14" s="2">
-        <v>6857.23</v>
-      </c>
-      <c r="G14" s="2">
-        <v>1.5</v>
-      </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="3">
         <v>2013</v>
       </c>
-      <c r="B15" s="2">
-        <v>400</v>
-      </c>
-      <c r="C15" s="2">
-        <v>4000</v>
-      </c>
-      <c r="E15" s="2">
-        <v>1690.355</v>
-      </c>
-      <c r="G15" s="2">
-        <v>30</v>
-      </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="3">
         <v>2014</v>
       </c>
-      <c r="E16" s="2">
-        <v>2255.857</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+    </row>
+    <row r="17" spans="1:1">
       <c r="A17" s="3">
         <v>2015</v>
       </c>
-      <c r="D17" s="2">
-        <v>248</v>
-      </c>
-      <c r="E17" s="2">
-        <v>1443.925</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+    </row>
+    <row r="18" spans="1:1">
       <c r="A18" s="3">
         <v>2016</v>
       </c>
-      <c r="E18" s="2">
-        <v>1664.465</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+    </row>
+    <row r="19" spans="1:1">
       <c r="A19" s="3">
         <v>2017</v>
       </c>
-      <c r="C19" s="2">
-        <v>100</v>
-      </c>
-      <c r="E19" s="2">
-        <v>4970.52</v>
-      </c>
-      <c r="F19" s="2">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+    </row>
+    <row r="20" spans="1:1">
       <c r="A20" s="3">
         <v>2018</v>
       </c>
-      <c r="D20" s="2">
-        <v>15036</v>
-      </c>
-      <c r="E20" s="2">
-        <v>2583.925</v>
-      </c>
-      <c r="G20" s="2">
-        <v>4500</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
+    </row>
+    <row r="21" spans="1:1">
       <c r="A21" s="3">
         <v>2019</v>
       </c>
-      <c r="C21" s="2">
-        <v>250</v>
-      </c>
-      <c r="E21" s="2">
-        <v>15187.31</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
+    </row>
+    <row r="22" spans="1:1">
       <c r="A22" s="3">
         <v>2020</v>
       </c>
-      <c r="C22" s="2">
-        <v>600</v>
-      </c>
-      <c r="E22" s="2">
-        <v>5012.295</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
+    </row>
+    <row r="23" spans="1:1">
       <c r="A23" s="3">
         <v>2021</v>
       </c>
-      <c r="C23" s="2">
-        <v>78.28</v>
-      </c>
-      <c r="E23" s="2">
-        <v>8628.021999999999</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
+    </row>
+    <row r="24" spans="1:1">
       <c r="A24" s="3">
         <v>2022</v>
       </c>
-      <c r="C24" s="2">
-        <v>142.76</v>
-      </c>
-      <c r="E24" s="2">
-        <v>10548.826</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
+    </row>
+    <row r="25" spans="1:1">
       <c r="A25" s="3">
         <v>2023</v>
       </c>
-      <c r="C25" s="2">
-        <v>438.67</v>
-      </c>
-      <c r="D25" s="2">
-        <v>4804</v>
-      </c>
-      <c r="E25" s="2">
-        <v>23815.572</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
+    </row>
+    <row r="26" spans="1:1">
       <c r="A26" s="3">
         <v>2024</v>
-      </c>
-      <c r="C26" s="2">
-        <v>1657.24</v>
-      </c>
-      <c r="E26" s="2">
-        <v>20798.506</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correct rerun, issues with outputs
</commit_message>
<xml_diff>
--- a/output_data/charts/capacity-15-CountyRegion-M010000US001.xlsx
+++ b/output_data/charts/capacity-15-CountyRegion-M010000US001.xlsx
@@ -167,10 +167,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -245,16 +245,22 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$26</c:f>
+              <c:f>Sheet1!$B$2:$B$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
+                <c:pt idx="13">
+                  <c:v>400</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -283,10 +289,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -361,16 +367,46 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$2:$C$26</c:f>
+              <c:f>Sheet1!$C$2:$C$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
+                <c:pt idx="13">
+                  <c:v>4000</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>78.28</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>142.76</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>438.67</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1668.74</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>489.46</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -399,10 +435,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -477,16 +513,28 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$26</c:f>
+              <c:f>Sheet1!$D$2:$D$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
+                <c:pt idx="15">
+                  <c:v>248</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>15036</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>4804</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -515,10 +563,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -593,16 +641,82 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$2:$E$26</c:f>
+              <c:f>Sheet1!$E$2:$E$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
+                <c:pt idx="5">
+                  <c:v>1.65</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>13.86</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>32.65</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>69.3</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>77.40000000000001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>518.3100000000001</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1817.347</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>6857.23</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1650.355</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2255.857</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1468.115</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1664.465</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5091.62</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2578.925</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>15198.51</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>5002.375</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>8620.972</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>10548.826</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23851.512</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>21017.826</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>15734.406</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -631,10 +745,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -709,16 +823,22 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$2:$F$26</c:f>
+              <c:f>Sheet1!$F$2:$F$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
+                <c:pt idx="17">
+                  <c:v>3500</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -747,10 +867,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -825,16 +945,52 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$2:$G$26</c:f>
+              <c:f>Sheet1!$G$2:$G$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>47.8</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>161.8</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.4</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>4500</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1264,7 +1420,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
@@ -1303,11 +1459,17 @@
       <c r="A2" s="3">
         <v>2000</v>
       </c>
+      <c r="G2" s="2">
+        <v>10</v>
+      </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3">
         <v>2001</v>
       </c>
+      <c r="G3" s="2">
+        <v>18</v>
+      </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="3">
@@ -1323,105 +1485,242 @@
       <c r="A6" s="3">
         <v>2004</v>
       </c>
+      <c r="G6" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="3">
         <v>2005</v>
       </c>
+      <c r="E7" s="2">
+        <v>1.65</v>
+      </c>
+      <c r="G7" s="2">
+        <v>8</v>
+      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="3">
         <v>2006</v>
       </c>
+      <c r="E8" s="2">
+        <v>13.86</v>
+      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="3">
         <v>2007</v>
       </c>
+      <c r="E9" s="2">
+        <v>32.65</v>
+      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="3">
         <v>2008</v>
       </c>
+      <c r="E10" s="2">
+        <v>69.3</v>
+      </c>
+      <c r="G10" s="2">
+        <v>1.8</v>
+      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="3">
         <v>2009</v>
       </c>
+      <c r="E11" s="2">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="G11" s="2">
+        <v>47.8</v>
+      </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="3">
         <v>2010</v>
       </c>
+      <c r="E12" s="2">
+        <v>518.3100000000001</v>
+      </c>
+      <c r="G12" s="2">
+        <v>161.8</v>
+      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="3">
         <v>2011</v>
       </c>
+      <c r="E13" s="2">
+        <v>1817.347</v>
+      </c>
+      <c r="G13" s="2">
+        <v>2.4</v>
+      </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="3">
         <v>2012</v>
       </c>
+      <c r="E14" s="2">
+        <v>6857.23</v>
+      </c>
+      <c r="G14" s="2">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="3">
         <v>2013</v>
       </c>
+      <c r="B15" s="2">
+        <v>400</v>
+      </c>
+      <c r="C15" s="2">
+        <v>4000</v>
+      </c>
+      <c r="E15" s="2">
+        <v>1650.355</v>
+      </c>
+      <c r="G15" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="3">
         <v>2014</v>
       </c>
-    </row>
-    <row r="17" spans="1:1">
+      <c r="E16" s="2">
+        <v>2255.857</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" s="3">
         <v>2015</v>
       </c>
-    </row>
-    <row r="18" spans="1:1">
+      <c r="D17" s="2">
+        <v>248</v>
+      </c>
+      <c r="E17" s="2">
+        <v>1468.115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" s="3">
         <v>2016</v>
       </c>
-    </row>
-    <row r="19" spans="1:1">
+      <c r="E18" s="2">
+        <v>1664.465</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
       <c r="A19" s="3">
         <v>2017</v>
       </c>
-    </row>
-    <row r="20" spans="1:1">
+      <c r="C19" s="2">
+        <v>100</v>
+      </c>
+      <c r="E19" s="2">
+        <v>5091.62</v>
+      </c>
+      <c r="F19" s="2">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" s="3">
         <v>2018</v>
       </c>
-    </row>
-    <row r="21" spans="1:1">
+      <c r="D20" s="2">
+        <v>15036</v>
+      </c>
+      <c r="E20" s="2">
+        <v>2578.925</v>
+      </c>
+      <c r="G20" s="2">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" s="3">
         <v>2019</v>
       </c>
-    </row>
-    <row r="22" spans="1:1">
+      <c r="C21" s="2">
+        <v>250</v>
+      </c>
+      <c r="E21" s="2">
+        <v>15198.51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" s="3">
         <v>2020</v>
       </c>
-    </row>
-    <row r="23" spans="1:1">
+      <c r="C22" s="2">
+        <v>600</v>
+      </c>
+      <c r="E22" s="2">
+        <v>5002.375</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
       <c r="A23" s="3">
         <v>2021</v>
       </c>
-    </row>
-    <row r="24" spans="1:1">
+      <c r="C23" s="2">
+        <v>78.28</v>
+      </c>
+      <c r="E23" s="2">
+        <v>8620.972</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" s="3">
         <v>2022</v>
       </c>
-    </row>
-    <row r="25" spans="1:1">
+      <c r="C24" s="2">
+        <v>142.76</v>
+      </c>
+      <c r="E24" s="2">
+        <v>10548.826</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" s="3">
         <v>2023</v>
       </c>
-    </row>
-    <row r="26" spans="1:1">
+      <c r="C25" s="2">
+        <v>438.67</v>
+      </c>
+      <c r="D25" s="2">
+        <v>4804</v>
+      </c>
+      <c r="E25" s="2">
+        <v>23851.512</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" s="3">
         <v>2024</v>
+      </c>
+      <c r="C26" s="2">
+        <v>1668.74</v>
+      </c>
+      <c r="E26" s="2">
+        <v>21017.826</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="3">
+        <v>2025</v>
+      </c>
+      <c r="C27" s="2">
+        <v>489.46</v>
+      </c>
+      <c r="E27" s="2">
+        <v>15734.406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data to include 2025.  Include non-member communities.
</commit_message>
<xml_diff>
--- a/output_data/charts/capacity-15-CountyRegion-M010000US001.xlsx
+++ b/output_data/charts/capacity-15-CountyRegion-M010000US001.xlsx
@@ -131,7 +131,8 @@
               <a:rPr lang="en-US" sz="1400" baseline="0">
                 <a:latin typeface="Arial"/>
               </a:rPr>
-              <a:t>Distributed Energy Resources Capacity by Year Opened - 15-County Region</a:t>
+              <a:t>Distributed Energy Resources Capacity by Year Opened -
+15-County Region</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -167,10 +168,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -245,16 +246,19 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$26</c:f>
+              <c:f>Sheet1!$B$2:$B$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="13">
                   <c:v>400</c:v>
                 </c:pt>
@@ -286,10 +290,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -364,16 +368,19 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$2:$C$26</c:f>
+              <c:f>Sheet1!$C$2:$C$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="13">
                   <c:v>4000</c:v>
                 </c:pt>
@@ -396,7 +403,10 @@
                   <c:v>438.67</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1657.24</c:v>
+                  <c:v>1668.74</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>489.46</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -426,10 +436,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -504,16 +514,19 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$26</c:f>
+              <c:f>Sheet1!$D$2:$D$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="15">
                   <c:v>248</c:v>
                 </c:pt>
@@ -551,10 +564,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -629,16 +642,19 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$2:$E$26</c:f>
+              <c:f>Sheet1!$E$2:$E$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="5">
                   <c:v>1.65</c:v>
                 </c:pt>
@@ -655,7 +671,7 @@
                   <c:v>77.40000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>515.23</c:v>
+                  <c:v>518.3100000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>1817.347</c:v>
@@ -664,40 +680,43 @@
                   <c:v>6857.23</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1690.355</c:v>
+                  <c:v>1650.355</c:v>
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>2255.857</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1443.925</c:v>
+                  <c:v>1468.115</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>1664.465</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4970.52</c:v>
+                  <c:v>5091.62</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2583.925</c:v>
+                  <c:v>2578.925</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>15187.31</c:v>
+                  <c:v>15198.51</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>5012.295</c:v>
+                  <c:v>5002.375</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>8628.021999999999</c:v>
+                  <c:v>8620.972</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>10548.826</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>23815.572</c:v>
+                  <c:v>23851.512</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>20798.506</c:v>
+                  <c:v>21017.826</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>15734.406</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -727,10 +746,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -805,16 +824,19 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$2:$F$26</c:f>
+              <c:f>Sheet1!$F$2:$F$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="17">
                   <c:v>3500</c:v>
                 </c:pt>
@@ -846,10 +868,10 @@
           </c:spPr>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$26</c:f>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>2000</c:v>
                 </c:pt>
@@ -924,16 +946,19 @@
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$2:$G$26</c:f>
+              <c:f>Sheet1!$G$2:$G$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
+                <c:ptCount val="26"/>
                 <c:pt idx="0">
                   <c:v>10</c:v>
                 </c:pt>
@@ -1396,7 +1421,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
@@ -1519,7 +1544,7 @@
         <v>2010</v>
       </c>
       <c r="E12" s="2">
-        <v>515.23</v>
+        <v>518.3100000000001</v>
       </c>
       <c r="G12" s="2">
         <v>161.8</v>
@@ -1558,7 +1583,7 @@
         <v>4000</v>
       </c>
       <c r="E15" s="2">
-        <v>1690.355</v>
+        <v>1650.355</v>
       </c>
       <c r="G15" s="2">
         <v>30</v>
@@ -1580,7 +1605,7 @@
         <v>248</v>
       </c>
       <c r="E17" s="2">
-        <v>1443.925</v>
+        <v>1468.115</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1599,7 +1624,7 @@
         <v>100</v>
       </c>
       <c r="E19" s="2">
-        <v>4970.52</v>
+        <v>5091.62</v>
       </c>
       <c r="F19" s="2">
         <v>3500</v>
@@ -1613,7 +1638,7 @@
         <v>15036</v>
       </c>
       <c r="E20" s="2">
-        <v>2583.925</v>
+        <v>2578.925</v>
       </c>
       <c r="G20" s="2">
         <v>4500</v>
@@ -1627,7 +1652,7 @@
         <v>250</v>
       </c>
       <c r="E21" s="2">
-        <v>15187.31</v>
+        <v>15198.51</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1638,7 +1663,7 @@
         <v>600</v>
       </c>
       <c r="E22" s="2">
-        <v>5012.295</v>
+        <v>5002.375</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1649,7 +1674,7 @@
         <v>78.28</v>
       </c>
       <c r="E23" s="2">
-        <v>8628.021999999999</v>
+        <v>8620.972</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1674,7 +1699,7 @@
         <v>4804</v>
       </c>
       <c r="E25" s="2">
-        <v>23815.572</v>
+        <v>23851.512</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1682,10 +1707,21 @@
         <v>2024</v>
       </c>
       <c r="C26" s="2">
-        <v>1657.24</v>
+        <v>1668.74</v>
       </c>
       <c r="E26" s="2">
-        <v>20798.506</v>
+        <v>21017.826</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="3">
+        <v>2025</v>
+      </c>
+      <c r="C27" s="2">
+        <v>489.46</v>
+      </c>
+      <c r="E27" s="2">
+        <v>15734.406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>